<commit_message>
Fix dashboard case status display
</commit_message>
<xml_diff>
--- a/cases.xlsx
+++ b/cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARUNA KUMARI\case-monitoring-devops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE567C4-E365-46D6-B34A-C604B43FB38E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53FD300F-CF8D-48FC-AF19-8BCF68688313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E980EED0-0792-47E1-B857-4595088FDCDC}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11835" xr2:uid="{E980EED0-0792-47E1-B857-4595088FDCDC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="27">
   <si>
     <t>Case Number</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>CS00121</t>
-  </si>
-  <si>
-    <t>CS00122</t>
   </si>
 </sst>
 </file>
@@ -738,24 +735,12 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="5">
-        <v>46299.791666666664</v>
-      </c>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>